<commit_message>
roand 2 xoa data
</commit_message>
<xml_diff>
--- a/CHITIEU/INPUT/DP.xlsx
+++ b/CHITIEU/INPUT/DP.xlsx
@@ -981,35 +981,20 @@
           <t>Xã Chiên Đàn</t>
         </is>
       </c>
-      <c r="D3" s="5">
-        <v>120</v>
-      </c>
-      <c r="E3" s="19">
-        <v>10</v>
-      </c>
+      <c r="D3" s="5"/>
+      <c r="E3" s="19"/>
       <c r="F3" s="6">
         <f>D3+E3</f>
-        <v>130</v>
-      </c>
-      <c r="G3" s="7">
-        <v>9854</v>
-      </c>
-      <c r="H3" s="19">
-        <v>10</v>
-      </c>
+      </c>
+      <c r="G3" s="7"/>
+      <c r="H3" s="19"/>
       <c r="I3" s="7">
         <f>G3+H3</f>
-        <v>9864</v>
-      </c>
-      <c r="J3" s="7">
-        <v>28186</v>
-      </c>
-      <c r="K3" s="19">
-        <v>10</v>
-      </c>
+      </c>
+      <c r="J3" s="7"/>
+      <c r="K3" s="19"/>
       <c r="L3" s="7">
         <f>J3+K3</f>
-        <v>28196</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
@@ -1028,35 +1013,20 @@
           <t>Xã Phú Ninh</t>
         </is>
       </c>
-      <c r="D4" s="5">
-        <v>67</v>
-      </c>
-      <c r="E4" s="19">
-        <v>10</v>
-      </c>
+      <c r="D4" s="5"/>
+      <c r="E4" s="19"/>
       <c r="F4" s="6">
         <f t="shared" ref="F4:F67" si="0">D4+E4</f>
-        <v>77</v>
-      </c>
-      <c r="G4" s="7">
-        <v>25287</v>
-      </c>
-      <c r="H4" s="19">
-        <v>10</v>
-      </c>
+      </c>
+      <c r="G4" s="7"/>
+      <c r="H4" s="19"/>
       <c r="I4" s="7">
         <f t="shared" ref="I4:I67" si="1">G4+H4</f>
-        <v>25297</v>
-      </c>
-      <c r="J4" s="7">
-        <v>9776</v>
-      </c>
-      <c r="K4" s="19">
-        <v>10</v>
-      </c>
+      </c>
+      <c r="J4" s="7"/>
+      <c r="K4" s="19"/>
       <c r="L4" s="7">
         <f t="shared" ref="L4:L67" si="2">J4+K4</f>
-        <v>9786</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
@@ -1075,33 +1045,15 @@
           <t>Xã Tây Hồ</t>
         </is>
       </c>
-      <c r="D5" s="5">
-        <v>177</v>
-      </c>
-      <c r="E5" s="19">
-        <v>10</v>
-      </c>
-      <c r="F5" s="6">
-        <v>177</v>
-      </c>
-      <c r="G5" s="7">
-        <v>12082</v>
-      </c>
-      <c r="H5" s="19">
-        <v>10</v>
-      </c>
-      <c r="I5" s="7">
-        <v>12082</v>
-      </c>
-      <c r="J5" s="7">
-        <v>12251</v>
-      </c>
-      <c r="K5" s="19">
-        <v>10</v>
-      </c>
-      <c r="L5" s="7">
-        <v>12251</v>
-      </c>
+      <c r="D5" s="5"/>
+      <c r="E5" s="19"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="7"/>
+      <c r="H5" s="19"/>
+      <c r="I5" s="7"/>
+      <c r="J5" s="7"/>
+      <c r="K5" s="19"/>
+      <c r="L5" s="7"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="inlineStr">
@@ -1119,29 +1071,15 @@
           <t>Xã A Vương</t>
         </is>
       </c>
-      <c r="D6" s="5">
-        <v>43517</v>
-      </c>
-      <c r="E6" s="8">
-        <v>1500</v>
-      </c>
-      <c r="F6" s="6">
-        <v>45017</v>
-      </c>
-      <c r="G6" s="7">
-        <v>1402</v>
-      </c>
+      <c r="D6" s="5"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="6"/>
+      <c r="G6" s="7"/>
       <c r="H6" s="19"/>
-      <c r="I6" s="7">
-        <v>1402</v>
-      </c>
-      <c r="J6" s="7">
-        <v>1719</v>
-      </c>
+      <c r="I6" s="7"/>
+      <c r="J6" s="7"/>
       <c r="K6" s="19"/>
-      <c r="L6" s="7">
-        <v>1719</v>
-      </c>
+      <c r="L6" s="7"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="inlineStr">
@@ -1159,29 +1097,15 @@
           <t>Xã Hùng Sơn</t>
         </is>
       </c>
-      <c r="D7" s="5">
-        <v>56897</v>
-      </c>
-      <c r="E7" s="8">
-        <v>2000</v>
-      </c>
-      <c r="F7" s="6">
-        <v>58897</v>
-      </c>
-      <c r="G7" s="7">
-        <v>206</v>
-      </c>
+      <c r="D7" s="5"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="7"/>
       <c r="H7" s="19"/>
-      <c r="I7" s="7">
-        <v>206</v>
-      </c>
-      <c r="J7" s="7">
-        <v>2555</v>
-      </c>
+      <c r="I7" s="7"/>
+      <c r="J7" s="7"/>
       <c r="K7" s="19"/>
-      <c r="L7" s="7">
-        <v>2555</v>
-      </c>
+      <c r="L7" s="7"/>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="inlineStr">
@@ -1199,29 +1123,15 @@
           <t>Xã Tây Giang</t>
         </is>
       </c>
-      <c r="D8" s="5">
-        <v>51583</v>
-      </c>
-      <c r="E8" s="3">
-        <v>500</v>
-      </c>
-      <c r="F8" s="6">
-        <v>52083</v>
-      </c>
-      <c r="G8" s="7">
-        <v>2021</v>
-      </c>
+      <c r="D8" s="5"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="6"/>
+      <c r="G8" s="7"/>
       <c r="H8" s="19"/>
-      <c r="I8" s="7">
-        <v>2021</v>
-      </c>
-      <c r="J8" s="7">
-        <v>1240</v>
-      </c>
+      <c r="I8" s="7"/>
+      <c r="J8" s="7"/>
       <c r="K8" s="19"/>
-      <c r="L8" s="7">
-        <v>1240</v>
-      </c>
+      <c r="L8" s="7"/>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="inlineStr">
@@ -1239,33 +1149,15 @@
           <t>Xã Nam Trà My</t>
         </is>
       </c>
-      <c r="D9" s="5">
-        <v>10304</v>
-      </c>
-      <c r="E9" s="3">
-        <v>100</v>
-      </c>
-      <c r="F9" s="6">
-        <v>10404</v>
-      </c>
-      <c r="G9" s="7">
-        <v>5015</v>
-      </c>
-      <c r="H9" s="3">
-        <v>100</v>
-      </c>
-      <c r="I9" s="7">
-        <v>5115</v>
-      </c>
-      <c r="J9" s="7">
-        <v>6793</v>
-      </c>
-      <c r="K9" s="3">
-        <v>100</v>
-      </c>
-      <c r="L9" s="7">
-        <v>6893</v>
-      </c>
+      <c r="D9" s="5"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="7"/>
+      <c r="J9" s="7"/>
+      <c r="K9" s="3"/>
+      <c r="L9" s="7"/>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="inlineStr">
@@ -1283,33 +1175,15 @@
           <t>Xã Trà Leng</t>
         </is>
       </c>
-      <c r="D10" s="5">
-        <v>10279</v>
-      </c>
-      <c r="E10" s="3">
-        <v>100</v>
-      </c>
-      <c r="F10" s="6">
-        <v>10379</v>
-      </c>
-      <c r="G10" s="7">
-        <v>68</v>
-      </c>
-      <c r="H10" s="3">
-        <v>50</v>
-      </c>
-      <c r="I10" s="7">
-        <v>118</v>
-      </c>
-      <c r="J10" s="7">
-        <v>2434</v>
-      </c>
-      <c r="K10" s="3">
-        <v>100</v>
-      </c>
-      <c r="L10" s="7">
-        <v>2534</v>
-      </c>
+      <c r="D10" s="5"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="7"/>
+      <c r="J10" s="7"/>
+      <c r="K10" s="3"/>
+      <c r="L10" s="7"/>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="inlineStr">
@@ -1327,31 +1201,15 @@
           <t>Xã Trà Linh</t>
         </is>
       </c>
-      <c r="D11" s="5">
-        <v>9049</v>
-      </c>
-      <c r="E11" s="3">
-        <v>100</v>
-      </c>
-      <c r="F11" s="6">
-        <v>9149</v>
-      </c>
-      <c r="G11" s="7">
-        <v>0</v>
-      </c>
+      <c r="D11" s="5"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="6"/>
+      <c r="G11" s="7"/>
       <c r="H11" s="19"/>
-      <c r="I11" s="7">
-        <v>0</v>
-      </c>
-      <c r="J11" s="7">
-        <v>4964</v>
-      </c>
-      <c r="K11" s="3">
-        <v>100</v>
-      </c>
-      <c r="L11" s="7">
-        <v>5064</v>
-      </c>
+      <c r="I11" s="7"/>
+      <c r="J11" s="7"/>
+      <c r="K11" s="3"/>
+      <c r="L11" s="7"/>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="inlineStr">
@@ -1369,33 +1227,15 @@
           <t>Xã Trà Tập</t>
         </is>
       </c>
-      <c r="D12" s="5">
-        <v>13169</v>
-      </c>
-      <c r="E12" s="3">
-        <v>150</v>
-      </c>
-      <c r="F12" s="6">
-        <v>13319</v>
-      </c>
-      <c r="G12" s="7">
-        <v>566</v>
-      </c>
-      <c r="H12" s="3">
-        <v>250</v>
-      </c>
-      <c r="I12" s="7">
-        <v>816</v>
-      </c>
-      <c r="J12" s="7">
-        <v>3782</v>
-      </c>
-      <c r="K12" s="3">
-        <v>100</v>
-      </c>
-      <c r="L12" s="7">
-        <v>3882</v>
-      </c>
+      <c r="D12" s="5"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="6"/>
+      <c r="G12" s="7"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="7"/>
+      <c r="J12" s="7"/>
+      <c r="K12" s="3"/>
+      <c r="L12" s="7"/>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="inlineStr">
@@ -1413,31 +1253,15 @@
           <t>Xã Trà Vân</t>
         </is>
       </c>
-      <c r="D13" s="5">
-        <v>14194</v>
-      </c>
-      <c r="E13" s="3">
-        <v>100</v>
-      </c>
-      <c r="F13" s="6">
-        <v>14294</v>
-      </c>
-      <c r="G13" s="7">
-        <v>0</v>
-      </c>
+      <c r="D13" s="5"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="6"/>
+      <c r="G13" s="7"/>
       <c r="H13" s="19"/>
-      <c r="I13" s="7">
-        <v>0</v>
-      </c>
-      <c r="J13" s="7">
-        <v>2937</v>
-      </c>
-      <c r="K13" s="3">
-        <v>100</v>
-      </c>
-      <c r="L13" s="7">
-        <v>3037</v>
-      </c>
+      <c r="I13" s="7"/>
+      <c r="J13" s="7"/>
+      <c r="K13" s="3"/>
+      <c r="L13" s="7"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="inlineStr">
@@ -1455,27 +1279,15 @@
           <t>Phường An Thắng</t>
         </is>
       </c>
-      <c r="D14" s="5">
-        <v>95</v>
-      </c>
+      <c r="D14" s="5"/>
       <c r="E14" s="19"/>
-      <c r="F14" s="6">
-        <v>95</v>
-      </c>
-      <c r="G14" s="7">
-        <v>32240</v>
-      </c>
+      <c r="F14" s="6"/>
+      <c r="G14" s="7"/>
       <c r="H14" s="19"/>
-      <c r="I14" s="7">
-        <v>32240</v>
-      </c>
-      <c r="J14" s="7">
-        <v>44235</v>
-      </c>
+      <c r="I14" s="7"/>
+      <c r="J14" s="7"/>
       <c r="K14" s="19"/>
-      <c r="L14" s="7">
-        <v>44235</v>
-      </c>
+      <c r="L14" s="7"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="inlineStr">
@@ -1493,27 +1305,15 @@
           <t>Xã Gò Nổi</t>
         </is>
       </c>
-      <c r="D15" s="5">
-        <v>47</v>
-      </c>
+      <c r="D15" s="5"/>
       <c r="E15" s="19"/>
-      <c r="F15" s="6">
-        <v>47</v>
-      </c>
-      <c r="G15" s="7">
-        <v>36809</v>
-      </c>
+      <c r="F15" s="6"/>
+      <c r="G15" s="7"/>
       <c r="H15" s="19"/>
-      <c r="I15" s="7">
-        <v>36809</v>
-      </c>
-      <c r="J15" s="7">
-        <v>13608</v>
-      </c>
+      <c r="I15" s="7"/>
+      <c r="J15" s="7"/>
       <c r="K15" s="19"/>
-      <c r="L15" s="7">
-        <v>13608</v>
-      </c>
+      <c r="L15" s="7"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="inlineStr">
@@ -1531,27 +1331,15 @@
           <t>Phường Điện Bàn</t>
         </is>
       </c>
-      <c r="D16" s="5">
-        <v>9</v>
-      </c>
+      <c r="D16" s="5"/>
       <c r="E16" s="19"/>
-      <c r="F16" s="6">
-        <v>9</v>
-      </c>
-      <c r="G16" s="7">
-        <v>25</v>
-      </c>
+      <c r="F16" s="6"/>
+      <c r="G16" s="7"/>
       <c r="H16" s="19"/>
-      <c r="I16" s="7">
-        <v>25</v>
-      </c>
-      <c r="J16" s="7">
-        <v>374</v>
-      </c>
+      <c r="I16" s="7"/>
+      <c r="J16" s="7"/>
       <c r="K16" s="19"/>
-      <c r="L16" s="7">
-        <v>374</v>
-      </c>
+      <c r="L16" s="7"/>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="inlineStr">
@@ -1569,27 +1357,15 @@
           <t>Phường Điện Bàn Bắc</t>
         </is>
       </c>
-      <c r="D17" s="5">
-        <v>0</v>
-      </c>
+      <c r="D17" s="5"/>
       <c r="E17" s="19"/>
-      <c r="F17" s="6">
-        <v>0</v>
-      </c>
-      <c r="G17" s="7">
-        <v>7885</v>
-      </c>
+      <c r="F17" s="6"/>
+      <c r="G17" s="7"/>
       <c r="H17" s="19"/>
-      <c r="I17" s="7">
-        <v>7885</v>
-      </c>
-      <c r="J17" s="7">
-        <v>6280</v>
-      </c>
+      <c r="I17" s="7"/>
+      <c r="J17" s="7"/>
       <c r="K17" s="19"/>
-      <c r="L17" s="7">
-        <v>6280</v>
-      </c>
+      <c r="L17" s="7"/>
     </row>
     <row r="18" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="inlineStr">
@@ -1607,27 +1383,15 @@
           <t>Xã Điện Bàn Tây</t>
         </is>
       </c>
-      <c r="D18" s="5">
-        <v>38</v>
-      </c>
+      <c r="D18" s="5"/>
       <c r="E18" s="19"/>
-      <c r="F18" s="6">
-        <v>38</v>
-      </c>
-      <c r="G18" s="7">
-        <v>5367</v>
-      </c>
+      <c r="F18" s="6"/>
+      <c r="G18" s="7"/>
       <c r="H18" s="19"/>
-      <c r="I18" s="7">
-        <v>5367</v>
-      </c>
-      <c r="J18" s="7">
-        <v>51416</v>
-      </c>
+      <c r="I18" s="7"/>
+      <c r="J18" s="7"/>
       <c r="K18" s="19"/>
-      <c r="L18" s="7">
-        <v>51416</v>
-      </c>
+      <c r="L18" s="7"/>
     </row>
     <row r="19" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="inlineStr">
@@ -1645,27 +1409,15 @@
           <t>Phường Điện Bàn Đông</t>
         </is>
       </c>
-      <c r="D19" s="5">
-        <v>17</v>
-      </c>
+      <c r="D19" s="5"/>
       <c r="E19" s="19"/>
-      <c r="F19" s="6">
-        <v>17</v>
-      </c>
-      <c r="G19" s="7">
-        <v>730</v>
-      </c>
+      <c r="F19" s="6"/>
+      <c r="G19" s="7"/>
       <c r="H19" s="19"/>
-      <c r="I19" s="7">
-        <v>730</v>
-      </c>
-      <c r="J19" s="7">
-        <v>10502</v>
-      </c>
+      <c r="I19" s="7"/>
+      <c r="J19" s="7"/>
       <c r="K19" s="19"/>
-      <c r="L19" s="7">
-        <v>10502</v>
-      </c>
+      <c r="L19" s="7"/>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="inlineStr">
@@ -1683,33 +1435,15 @@
           <t>Xã Duy Nghĩa</t>
         </is>
       </c>
-      <c r="D20" s="5">
-        <v>702</v>
-      </c>
-      <c r="E20" s="3">
-        <v>-100</v>
-      </c>
-      <c r="F20" s="6">
-        <v>602</v>
-      </c>
-      <c r="G20" s="7">
-        <v>17182</v>
-      </c>
-      <c r="H20" s="8">
-        <v>-1078</v>
-      </c>
-      <c r="I20" s="7">
-        <v>16104</v>
-      </c>
-      <c r="J20" s="7">
-        <v>890</v>
-      </c>
-      <c r="K20" s="3">
-        <v>-300</v>
-      </c>
-      <c r="L20" s="7">
-        <v>590</v>
-      </c>
+      <c r="D20" s="5"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="6"/>
+      <c r="G20" s="7"/>
+      <c r="H20" s="8"/>
+      <c r="I20" s="7"/>
+      <c r="J20" s="7"/>
+      <c r="K20" s="3"/>
+      <c r="L20" s="7"/>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="inlineStr">
@@ -1727,31 +1461,15 @@
           <t>Xã Nam Phước</t>
         </is>
       </c>
-      <c r="D21" s="5">
-        <v>598</v>
-      </c>
+      <c r="D21" s="5"/>
       <c r="E21" s="19"/>
-      <c r="F21" s="6">
-        <v>598</v>
-      </c>
-      <c r="G21" s="7">
-        <v>36670</v>
-      </c>
-      <c r="H21" s="8">
-        <v>-2000</v>
-      </c>
-      <c r="I21" s="7">
-        <v>34670</v>
-      </c>
-      <c r="J21" s="7">
-        <v>933</v>
-      </c>
-      <c r="K21" s="3">
-        <v>-300</v>
-      </c>
-      <c r="L21" s="7">
-        <v>633</v>
-      </c>
+      <c r="F21" s="6"/>
+      <c r="G21" s="7"/>
+      <c r="H21" s="8"/>
+      <c r="I21" s="7"/>
+      <c r="J21" s="7"/>
+      <c r="K21" s="3"/>
+      <c r="L21" s="7"/>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="inlineStr">
@@ -1769,31 +1487,15 @@
           <t>Xã Duy Xuyên</t>
         </is>
       </c>
-      <c r="D22" s="5">
-        <v>105</v>
-      </c>
+      <c r="D22" s="5"/>
       <c r="E22" s="19"/>
-      <c r="F22" s="6">
-        <v>105</v>
-      </c>
-      <c r="G22" s="7">
-        <v>14107</v>
-      </c>
-      <c r="H22" s="3">
-        <v>-600</v>
-      </c>
-      <c r="I22" s="7">
-        <v>13507</v>
-      </c>
-      <c r="J22" s="7">
-        <v>1255</v>
-      </c>
-      <c r="K22" s="3">
-        <v>-400</v>
-      </c>
-      <c r="L22" s="7">
-        <v>855</v>
-      </c>
+      <c r="F22" s="6"/>
+      <c r="G22" s="7"/>
+      <c r="H22" s="3"/>
+      <c r="I22" s="7"/>
+      <c r="J22" s="7"/>
+      <c r="K22" s="3"/>
+      <c r="L22" s="7"/>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="inlineStr">
@@ -1811,33 +1513,15 @@
           <t>Xã Thu Bồn</t>
         </is>
       </c>
-      <c r="D23" s="5">
-        <v>1007</v>
-      </c>
-      <c r="E23" s="3">
-        <v>-300</v>
-      </c>
-      <c r="F23" s="6">
-        <v>707</v>
-      </c>
-      <c r="G23" s="7">
-        <v>39339</v>
-      </c>
-      <c r="H23" s="8">
-        <v>-3795</v>
-      </c>
-      <c r="I23" s="7">
-        <v>35544</v>
-      </c>
-      <c r="J23" s="7">
-        <v>3592</v>
-      </c>
-      <c r="K23" s="8">
-        <v>-1000</v>
-      </c>
-      <c r="L23" s="7">
-        <v>2592</v>
-      </c>
+      <c r="D23" s="5"/>
+      <c r="E23" s="3"/>
+      <c r="F23" s="6"/>
+      <c r="G23" s="7"/>
+      <c r="H23" s="8"/>
+      <c r="I23" s="7"/>
+      <c r="J23" s="7"/>
+      <c r="K23" s="8"/>
+      <c r="L23" s="7"/>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="inlineStr">
@@ -1855,33 +1539,15 @@
           <t>Xã Thăng An</t>
         </is>
       </c>
-      <c r="D24" s="5">
-        <v>1230</v>
-      </c>
-      <c r="E24" s="3">
-        <v>-10</v>
-      </c>
-      <c r="F24" s="6">
-        <v>1220</v>
-      </c>
-      <c r="G24" s="7">
-        <v>78264</v>
-      </c>
-      <c r="H24" s="8">
-        <v>-3000</v>
-      </c>
-      <c r="I24" s="7">
-        <v>75264</v>
-      </c>
-      <c r="J24" s="7">
-        <v>8040</v>
-      </c>
-      <c r="K24" s="8">
-        <v>-1500</v>
-      </c>
-      <c r="L24" s="7">
-        <v>6540</v>
-      </c>
+      <c r="D24" s="5"/>
+      <c r="E24" s="3"/>
+      <c r="F24" s="6"/>
+      <c r="G24" s="7"/>
+      <c r="H24" s="8"/>
+      <c r="I24" s="7"/>
+      <c r="J24" s="7"/>
+      <c r="K24" s="8"/>
+      <c r="L24" s="7"/>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="inlineStr">
@@ -1899,33 +1565,15 @@
           <t>Xã Thăng Bình</t>
         </is>
       </c>
-      <c r="D25" s="5">
-        <v>625</v>
-      </c>
-      <c r="E25" s="3">
-        <v>-10</v>
-      </c>
-      <c r="F25" s="6">
-        <v>615</v>
-      </c>
-      <c r="G25" s="7">
-        <v>103865</v>
-      </c>
-      <c r="H25" s="8">
-        <v>-5000</v>
-      </c>
-      <c r="I25" s="7">
-        <v>98865</v>
-      </c>
-      <c r="J25" s="7">
-        <v>16201</v>
-      </c>
-      <c r="K25" s="8">
-        <v>-1500</v>
-      </c>
-      <c r="L25" s="7">
-        <v>14701</v>
-      </c>
+      <c r="D25" s="5"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="6"/>
+      <c r="G25" s="7"/>
+      <c r="H25" s="8"/>
+      <c r="I25" s="7"/>
+      <c r="J25" s="7"/>
+      <c r="K25" s="8"/>
+      <c r="L25" s="7"/>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="inlineStr">
@@ -1943,33 +1591,15 @@
           <t>Xã Thăng Phú</t>
         </is>
       </c>
-      <c r="D26" s="5">
-        <v>313</v>
-      </c>
-      <c r="E26" s="3">
-        <v>-10</v>
-      </c>
-      <c r="F26" s="6">
-        <v>303</v>
-      </c>
-      <c r="G26" s="7">
-        <v>61520</v>
-      </c>
-      <c r="H26" s="8">
-        <v>-4000</v>
-      </c>
-      <c r="I26" s="7">
-        <v>57520</v>
-      </c>
-      <c r="J26" s="7">
-        <v>2668</v>
-      </c>
-      <c r="K26" s="3">
-        <v>-500</v>
-      </c>
-      <c r="L26" s="7">
-        <v>2168</v>
-      </c>
+      <c r="D26" s="5"/>
+      <c r="E26" s="3"/>
+      <c r="F26" s="6"/>
+      <c r="G26" s="7"/>
+      <c r="H26" s="8"/>
+      <c r="I26" s="7"/>
+      <c r="J26" s="7"/>
+      <c r="K26" s="3"/>
+      <c r="L26" s="7"/>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="inlineStr">
@@ -1987,33 +1617,15 @@
           <t>Xã Thăng Trường</t>
         </is>
       </c>
-      <c r="D27" s="5">
-        <v>376</v>
-      </c>
-      <c r="E27" s="3">
-        <v>-10</v>
-      </c>
-      <c r="F27" s="6">
-        <v>366</v>
-      </c>
-      <c r="G27" s="7">
-        <v>25581</v>
-      </c>
-      <c r="H27" s="8">
-        <v>-3000</v>
-      </c>
-      <c r="I27" s="7">
-        <v>22581</v>
-      </c>
-      <c r="J27" s="7">
-        <v>5574</v>
-      </c>
-      <c r="K27" s="3">
-        <v>-500</v>
-      </c>
-      <c r="L27" s="7">
-        <v>5074</v>
-      </c>
+      <c r="D27" s="5"/>
+      <c r="E27" s="3"/>
+      <c r="F27" s="6"/>
+      <c r="G27" s="7"/>
+      <c r="H27" s="8"/>
+      <c r="I27" s="7"/>
+      <c r="J27" s="7"/>
+      <c r="K27" s="3"/>
+      <c r="L27" s="7"/>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="inlineStr">
@@ -2031,33 +1643,15 @@
           <t>Xã Thăng Điền</t>
         </is>
       </c>
-      <c r="D28" s="5">
-        <v>454</v>
-      </c>
-      <c r="E28" s="3">
-        <v>-10</v>
-      </c>
-      <c r="F28" s="6">
-        <v>444</v>
-      </c>
-      <c r="G28" s="7">
-        <v>90818</v>
-      </c>
-      <c r="H28" s="8">
-        <v>-5000</v>
-      </c>
-      <c r="I28" s="7">
-        <v>85818</v>
-      </c>
-      <c r="J28" s="7">
-        <v>10294</v>
-      </c>
-      <c r="K28" s="8">
-        <v>-1500</v>
-      </c>
-      <c r="L28" s="7">
-        <v>8794</v>
-      </c>
+      <c r="D28" s="5"/>
+      <c r="E28" s="3"/>
+      <c r="F28" s="6"/>
+      <c r="G28" s="7"/>
+      <c r="H28" s="8"/>
+      <c r="I28" s="7"/>
+      <c r="J28" s="7"/>
+      <c r="K28" s="8"/>
+      <c r="L28" s="7"/>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="inlineStr">
@@ -2075,33 +1669,15 @@
           <t>Xã Đồng Dương</t>
         </is>
       </c>
-      <c r="D29" s="5">
-        <v>578</v>
-      </c>
-      <c r="E29" s="3">
-        <v>-50</v>
-      </c>
-      <c r="F29" s="6">
-        <v>528</v>
-      </c>
-      <c r="G29" s="7">
-        <v>87729</v>
-      </c>
-      <c r="H29" s="8">
-        <v>-5000</v>
-      </c>
-      <c r="I29" s="7">
-        <v>82729</v>
-      </c>
-      <c r="J29" s="7">
-        <v>6338</v>
-      </c>
-      <c r="K29" s="8">
-        <v>-1500</v>
-      </c>
-      <c r="L29" s="7">
-        <v>4838</v>
-      </c>
+      <c r="D29" s="5"/>
+      <c r="E29" s="3"/>
+      <c r="F29" s="6"/>
+      <c r="G29" s="7"/>
+      <c r="H29" s="8"/>
+      <c r="I29" s="7"/>
+      <c r="J29" s="7"/>
+      <c r="K29" s="8"/>
+      <c r="L29" s="7"/>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="inlineStr">
@@ -2119,33 +1695,15 @@
           <t>Xã Nông Sơn</t>
         </is>
       </c>
-      <c r="D30" s="5">
-        <v>618</v>
-      </c>
-      <c r="E30" s="3">
-        <v>-100</v>
-      </c>
-      <c r="F30" s="6">
-        <v>518</v>
-      </c>
-      <c r="G30" s="9">
-        <v>12769</v>
-      </c>
-      <c r="H30" s="8">
-        <v>-1000</v>
-      </c>
-      <c r="I30" s="7">
-        <v>11769</v>
-      </c>
-      <c r="J30" s="7">
-        <v>8584</v>
-      </c>
-      <c r="K30" s="8">
-        <v>-1000</v>
-      </c>
-      <c r="L30" s="7">
-        <v>7584</v>
-      </c>
+      <c r="D30" s="5"/>
+      <c r="E30" s="3"/>
+      <c r="F30" s="6"/>
+      <c r="G30" s="9"/>
+      <c r="H30" s="8"/>
+      <c r="I30" s="7"/>
+      <c r="J30" s="7"/>
+      <c r="K30" s="8"/>
+      <c r="L30" s="7"/>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="inlineStr">
@@ -2163,33 +1721,15 @@
           <t>Xã Quế Phước</t>
         </is>
       </c>
-      <c r="D31" s="5">
-        <v>1051</v>
-      </c>
-      <c r="E31" s="3">
-        <v>-200</v>
-      </c>
-      <c r="F31" s="6">
-        <v>851</v>
-      </c>
-      <c r="G31" s="9">
-        <v>12633</v>
-      </c>
-      <c r="H31" s="8">
-        <v>-1000</v>
-      </c>
-      <c r="I31" s="7">
-        <v>11633</v>
-      </c>
-      <c r="J31" s="7">
-        <v>6567</v>
-      </c>
-      <c r="K31" s="8">
-        <v>-1000</v>
-      </c>
-      <c r="L31" s="7">
-        <v>5567</v>
-      </c>
+      <c r="D31" s="5"/>
+      <c r="E31" s="3"/>
+      <c r="F31" s="6"/>
+      <c r="G31" s="9"/>
+      <c r="H31" s="8"/>
+      <c r="I31" s="7"/>
+      <c r="J31" s="7"/>
+      <c r="K31" s="8"/>
+      <c r="L31" s="7"/>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="inlineStr">
@@ -2207,33 +1747,15 @@
           <t>Xã Quế Sơn</t>
         </is>
       </c>
-      <c r="D32" s="5">
-        <v>1715</v>
-      </c>
-      <c r="E32" s="3">
-        <v>-300</v>
-      </c>
-      <c r="F32" s="6">
-        <v>1415</v>
-      </c>
-      <c r="G32" s="9">
-        <v>67700</v>
-      </c>
-      <c r="H32" s="8">
-        <v>-2500</v>
-      </c>
-      <c r="I32" s="7">
-        <v>65200</v>
-      </c>
-      <c r="J32" s="7">
-        <v>21148</v>
-      </c>
-      <c r="K32" s="8">
-        <v>-3000</v>
-      </c>
-      <c r="L32" s="7">
-        <v>18148</v>
-      </c>
+      <c r="D32" s="5"/>
+      <c r="E32" s="3"/>
+      <c r="F32" s="6"/>
+      <c r="G32" s="9"/>
+      <c r="H32" s="8"/>
+      <c r="I32" s="7"/>
+      <c r="J32" s="7"/>
+      <c r="K32" s="8"/>
+      <c r="L32" s="7"/>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="inlineStr">
@@ -2251,33 +1773,15 @@
           <t>Xã Quế Sơn Trung</t>
         </is>
       </c>
-      <c r="D33" s="5">
-        <v>1967</v>
-      </c>
-      <c r="E33" s="3">
-        <v>-100</v>
-      </c>
-      <c r="F33" s="6">
-        <v>1867</v>
-      </c>
-      <c r="G33" s="9">
-        <v>108482</v>
-      </c>
-      <c r="H33" s="8">
-        <v>-2500</v>
-      </c>
-      <c r="I33" s="7">
-        <v>105982</v>
-      </c>
-      <c r="J33" s="7">
-        <v>30620</v>
-      </c>
-      <c r="K33" s="8">
-        <v>-3000</v>
-      </c>
-      <c r="L33" s="7">
-        <v>27620</v>
-      </c>
+      <c r="D33" s="5"/>
+      <c r="E33" s="3"/>
+      <c r="F33" s="6"/>
+      <c r="G33" s="9"/>
+      <c r="H33" s="8"/>
+      <c r="I33" s="7"/>
+      <c r="J33" s="7"/>
+      <c r="K33" s="8"/>
+      <c r="L33" s="7"/>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="inlineStr">
@@ -2295,33 +1799,15 @@
           <t>Xã Xuân Phú</t>
         </is>
       </c>
-      <c r="D34" s="5">
-        <v>298</v>
-      </c>
-      <c r="E34" s="3">
-        <v>-200</v>
-      </c>
-      <c r="F34" s="6">
-        <v>98</v>
-      </c>
-      <c r="G34" s="9">
-        <v>69668</v>
-      </c>
-      <c r="H34" s="8">
-        <v>-3000</v>
-      </c>
-      <c r="I34" s="7">
-        <v>66668</v>
-      </c>
-      <c r="J34" s="7">
-        <v>14148</v>
-      </c>
-      <c r="K34" s="8">
-        <v>-2000</v>
-      </c>
-      <c r="L34" s="7">
-        <v>12148</v>
-      </c>
+      <c r="D34" s="5"/>
+      <c r="E34" s="3"/>
+      <c r="F34" s="6"/>
+      <c r="G34" s="9"/>
+      <c r="H34" s="8"/>
+      <c r="I34" s="7"/>
+      <c r="J34" s="7"/>
+      <c r="K34" s="8"/>
+      <c r="L34" s="7"/>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="inlineStr">
@@ -2339,29 +1825,15 @@
           <t>Xã Trà Giáp</t>
         </is>
       </c>
-      <c r="D35" s="5">
-        <v>44246</v>
-      </c>
-      <c r="E35" s="8">
-        <v>1000</v>
-      </c>
-      <c r="F35" s="6">
-        <v>45246</v>
-      </c>
-      <c r="G35" s="7">
-        <v>294</v>
-      </c>
+      <c r="D35" s="5"/>
+      <c r="E35" s="8"/>
+      <c r="F35" s="6"/>
+      <c r="G35" s="7"/>
       <c r="H35" s="19"/>
-      <c r="I35" s="7">
-        <v>294</v>
-      </c>
-      <c r="J35" s="7">
-        <v>2576</v>
-      </c>
+      <c r="I35" s="7"/>
+      <c r="J35" s="7"/>
       <c r="K35" s="19"/>
-      <c r="L35" s="7">
-        <v>2576</v>
-      </c>
+      <c r="L35" s="7"/>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="inlineStr">
@@ -2379,29 +1851,15 @@
           <t>Xã Trà Liên</t>
         </is>
       </c>
-      <c r="D36" s="5">
-        <v>43498</v>
-      </c>
-      <c r="E36" s="8">
-        <v>1500</v>
-      </c>
-      <c r="F36" s="6">
-        <v>44998</v>
-      </c>
-      <c r="G36" s="7">
-        <v>9352</v>
-      </c>
+      <c r="D36" s="5"/>
+      <c r="E36" s="8"/>
+      <c r="F36" s="6"/>
+      <c r="G36" s="7"/>
       <c r="H36" s="19"/>
-      <c r="I36" s="7">
-        <v>9352</v>
-      </c>
-      <c r="J36" s="7">
-        <v>5042</v>
-      </c>
+      <c r="I36" s="7"/>
+      <c r="J36" s="7"/>
       <c r="K36" s="19"/>
-      <c r="L36" s="7">
-        <v>5042</v>
-      </c>
+      <c r="L36" s="7"/>
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="inlineStr">
@@ -2419,29 +1877,15 @@
           <t>Xã Trà My</t>
         </is>
       </c>
-      <c r="D37" s="5">
-        <v>34810</v>
-      </c>
-      <c r="E37" s="3">
-        <v>500</v>
-      </c>
-      <c r="F37" s="6">
-        <v>35310</v>
-      </c>
-      <c r="G37" s="7">
-        <v>16032</v>
-      </c>
+      <c r="D37" s="5"/>
+      <c r="E37" s="3"/>
+      <c r="F37" s="6"/>
+      <c r="G37" s="7"/>
       <c r="H37" s="19"/>
-      <c r="I37" s="7">
-        <v>16032</v>
-      </c>
-      <c r="J37" s="7">
-        <v>16017</v>
-      </c>
+      <c r="I37" s="7"/>
+      <c r="J37" s="7"/>
       <c r="K37" s="19"/>
-      <c r="L37" s="7">
-        <v>16017</v>
-      </c>
+      <c r="L37" s="7"/>
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="inlineStr">
@@ -2459,29 +1903,15 @@
           <t>Xã Trà Tân</t>
         </is>
       </c>
-      <c r="D38" s="5">
-        <v>26369</v>
-      </c>
-      <c r="E38" s="8">
-        <v>1000</v>
-      </c>
-      <c r="F38" s="6">
-        <v>27369</v>
-      </c>
-      <c r="G38" s="7">
-        <v>8279</v>
-      </c>
+      <c r="D38" s="5"/>
+      <c r="E38" s="8"/>
+      <c r="F38" s="6"/>
+      <c r="G38" s="7"/>
       <c r="H38" s="19"/>
-      <c r="I38" s="7">
-        <v>8279</v>
-      </c>
-      <c r="J38" s="7">
-        <v>4518</v>
-      </c>
+      <c r="I38" s="7"/>
+      <c r="J38" s="7"/>
       <c r="K38" s="19"/>
-      <c r="L38" s="7">
-        <v>4518</v>
-      </c>
+      <c r="L38" s="7"/>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="inlineStr">
@@ -2499,29 +1929,15 @@
           <t>Xã Trà Đốc</t>
         </is>
       </c>
-      <c r="D39" s="5">
-        <v>62174</v>
-      </c>
-      <c r="E39" s="8">
-        <v>1000</v>
-      </c>
-      <c r="F39" s="6">
-        <v>63174</v>
-      </c>
-      <c r="G39" s="7">
-        <v>36</v>
-      </c>
+      <c r="D39" s="5"/>
+      <c r="E39" s="8"/>
+      <c r="F39" s="6"/>
+      <c r="G39" s="7"/>
       <c r="H39" s="19"/>
-      <c r="I39" s="7">
-        <v>36</v>
-      </c>
-      <c r="J39" s="7">
-        <v>5096</v>
-      </c>
+      <c r="I39" s="7"/>
+      <c r="J39" s="7"/>
       <c r="K39" s="19"/>
-      <c r="L39" s="7">
-        <v>5096</v>
-      </c>
+      <c r="L39" s="7"/>
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="inlineStr">
@@ -2539,31 +1955,15 @@
           <t>Xã Hà Nha</t>
         </is>
       </c>
-      <c r="D40" s="5">
-        <v>153</v>
-      </c>
+      <c r="D40" s="5"/>
       <c r="E40" s="19"/>
-      <c r="F40" s="6">
-        <v>153</v>
-      </c>
-      <c r="G40" s="7">
-        <v>19776</v>
-      </c>
-      <c r="H40" s="3">
-        <v>-500</v>
-      </c>
-      <c r="I40" s="7">
-        <v>19276</v>
-      </c>
-      <c r="J40" s="7">
-        <v>23187</v>
-      </c>
-      <c r="K40" s="8">
-        <v>-4000</v>
-      </c>
-      <c r="L40" s="7">
-        <v>19187</v>
-      </c>
+      <c r="F40" s="6"/>
+      <c r="G40" s="7"/>
+      <c r="H40" s="3"/>
+      <c r="I40" s="7"/>
+      <c r="J40" s="7"/>
+      <c r="K40" s="8"/>
+      <c r="L40" s="7"/>
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="inlineStr">
@@ -2581,33 +1981,15 @@
           <t>Xã Phú Thuận</t>
         </is>
       </c>
-      <c r="D41" s="5">
-        <v>1970</v>
-      </c>
-      <c r="E41" s="8">
-        <v>-1000</v>
-      </c>
-      <c r="F41" s="6">
-        <v>970</v>
-      </c>
-      <c r="G41" s="7">
-        <v>8747</v>
-      </c>
-      <c r="H41" s="8">
-        <v>-2000</v>
-      </c>
-      <c r="I41" s="7">
-        <v>6747</v>
-      </c>
-      <c r="J41" s="7">
-        <v>14819</v>
-      </c>
-      <c r="K41" s="8">
-        <v>-2000</v>
-      </c>
-      <c r="L41" s="7">
-        <v>12819</v>
-      </c>
+      <c r="D41" s="5"/>
+      <c r="E41" s="8"/>
+      <c r="F41" s="6"/>
+      <c r="G41" s="7"/>
+      <c r="H41" s="8"/>
+      <c r="I41" s="7"/>
+      <c r="J41" s="7"/>
+      <c r="K41" s="8"/>
+      <c r="L41" s="7"/>
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="inlineStr">
@@ -2625,33 +2007,15 @@
           <t>Xã Thượng Đức</t>
         </is>
       </c>
-      <c r="D42" s="5">
-        <v>1799</v>
-      </c>
-      <c r="E42" s="8">
-        <v>-1500</v>
-      </c>
-      <c r="F42" s="6">
-        <v>299</v>
-      </c>
-      <c r="G42" s="7">
-        <v>15036</v>
-      </c>
-      <c r="H42" s="8">
-        <v>-1000</v>
-      </c>
-      <c r="I42" s="7">
-        <v>14036</v>
-      </c>
-      <c r="J42" s="7">
-        <v>15068</v>
-      </c>
-      <c r="K42" s="8">
-        <v>-1000</v>
-      </c>
-      <c r="L42" s="7">
-        <v>14068</v>
-      </c>
+      <c r="D42" s="5"/>
+      <c r="E42" s="8"/>
+      <c r="F42" s="6"/>
+      <c r="G42" s="7"/>
+      <c r="H42" s="8"/>
+      <c r="I42" s="7"/>
+      <c r="J42" s="7"/>
+      <c r="K42" s="8"/>
+      <c r="L42" s="7"/>
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="inlineStr">
@@ -2669,31 +2033,15 @@
           <t>Xã Vu Gia</t>
         </is>
       </c>
-      <c r="D43" s="5">
-        <v>160</v>
-      </c>
+      <c r="D43" s="5"/>
       <c r="E43" s="19"/>
-      <c r="F43" s="6">
-        <v>160</v>
-      </c>
-      <c r="G43" s="7">
-        <v>27568</v>
-      </c>
-      <c r="H43" s="3">
-        <v>-500</v>
-      </c>
-      <c r="I43" s="7">
-        <v>27068</v>
-      </c>
-      <c r="J43" s="7">
-        <v>10706</v>
-      </c>
-      <c r="K43" s="8">
-        <v>-6000</v>
-      </c>
-      <c r="L43" s="7">
-        <v>4706</v>
-      </c>
+      <c r="F43" s="6"/>
+      <c r="G43" s="7"/>
+      <c r="H43" s="3"/>
+      <c r="I43" s="7"/>
+      <c r="J43" s="7"/>
+      <c r="K43" s="8"/>
+      <c r="L43" s="7"/>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="inlineStr">
@@ -2711,29 +2059,15 @@
           <t>Xã Đại Lộc</t>
         </is>
       </c>
-      <c r="D44" s="5">
-        <v>10</v>
-      </c>
+      <c r="D44" s="5"/>
       <c r="E44" s="19"/>
-      <c r="F44" s="6">
-        <v>10</v>
-      </c>
-      <c r="G44" s="7">
-        <v>23679</v>
-      </c>
+      <c r="F44" s="6"/>
+      <c r="G44" s="7"/>
       <c r="H44" s="19"/>
-      <c r="I44" s="7">
-        <v>23679</v>
-      </c>
-      <c r="J44" s="7">
-        <v>40352</v>
-      </c>
-      <c r="K44" s="8">
-        <v>-7000</v>
-      </c>
-      <c r="L44" s="7">
-        <v>33352</v>
-      </c>
+      <c r="I44" s="7"/>
+      <c r="J44" s="7"/>
+      <c r="K44" s="8"/>
+      <c r="L44" s="7"/>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="inlineStr">
@@ -2751,33 +2085,15 @@
           <t>Xã Núi Thành</t>
         </is>
       </c>
-      <c r="D45" s="5">
-        <v>549</v>
-      </c>
-      <c r="E45" s="3">
-        <v>-15</v>
-      </c>
-      <c r="F45" s="6">
-        <v>534</v>
-      </c>
-      <c r="G45" s="7">
-        <v>991</v>
-      </c>
-      <c r="H45" s="3">
-        <v>-100</v>
-      </c>
-      <c r="I45" s="7">
-        <v>891</v>
-      </c>
-      <c r="J45" s="7">
-        <v>447</v>
-      </c>
-      <c r="K45" s="3">
-        <v>-50</v>
-      </c>
-      <c r="L45" s="7">
-        <v>397</v>
-      </c>
+      <c r="D45" s="5"/>
+      <c r="E45" s="3"/>
+      <c r="F45" s="6"/>
+      <c r="G45" s="7"/>
+      <c r="H45" s="3"/>
+      <c r="I45" s="7"/>
+      <c r="J45" s="7"/>
+      <c r="K45" s="3"/>
+      <c r="L45" s="7"/>
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="inlineStr">
@@ -2795,33 +2111,15 @@
           <t>Xã Tam Anh</t>
         </is>
       </c>
-      <c r="D46" s="5">
-        <v>143</v>
-      </c>
-      <c r="E46" s="3">
-        <v>-55</v>
-      </c>
-      <c r="F46" s="6">
-        <v>88</v>
-      </c>
-      <c r="G46" s="7">
-        <v>65279</v>
-      </c>
-      <c r="H46" s="8">
-        <v>-14000</v>
-      </c>
-      <c r="I46" s="7">
-        <v>51279</v>
-      </c>
-      <c r="J46" s="7">
-        <v>2527</v>
-      </c>
-      <c r="K46" s="8">
-        <v>-1650</v>
-      </c>
-      <c r="L46" s="7">
-        <v>877</v>
-      </c>
+      <c r="D46" s="5"/>
+      <c r="E46" s="3"/>
+      <c r="F46" s="6"/>
+      <c r="G46" s="7"/>
+      <c r="H46" s="8"/>
+      <c r="I46" s="7"/>
+      <c r="J46" s="7"/>
+      <c r="K46" s="8"/>
+      <c r="L46" s="7"/>
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="inlineStr">
@@ -2839,29 +2137,15 @@
           <t>Xã Tam Hải</t>
         </is>
       </c>
-      <c r="D47" s="5">
-        <v>90</v>
-      </c>
+      <c r="D47" s="5"/>
       <c r="E47" s="19"/>
-      <c r="F47" s="6">
-        <v>90</v>
-      </c>
-      <c r="G47" s="7">
-        <v>42309</v>
-      </c>
-      <c r="H47" s="8">
-        <v>-9850</v>
-      </c>
-      <c r="I47" s="7">
-        <v>32459</v>
-      </c>
-      <c r="J47" s="7">
-        <v>33</v>
-      </c>
+      <c r="F47" s="6"/>
+      <c r="G47" s="7"/>
+      <c r="H47" s="8"/>
+      <c r="I47" s="7"/>
+      <c r="J47" s="7"/>
       <c r="K47" s="19"/>
-      <c r="L47" s="7">
-        <v>33</v>
-      </c>
+      <c r="L47" s="7"/>
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="inlineStr">
@@ -2879,33 +2163,15 @@
           <t>Xã Tam Mỹ</t>
         </is>
       </c>
-      <c r="D48" s="5">
-        <v>1547</v>
-      </c>
-      <c r="E48" s="3">
-        <v>-480</v>
-      </c>
-      <c r="F48" s="6">
-        <v>1067</v>
-      </c>
-      <c r="G48" s="7">
-        <v>19336</v>
-      </c>
-      <c r="H48" s="8">
-        <v>-1000</v>
-      </c>
-      <c r="I48" s="7">
-        <v>18336</v>
-      </c>
-      <c r="J48" s="7">
-        <v>1924</v>
-      </c>
-      <c r="K48" s="3">
-        <v>-850</v>
-      </c>
-      <c r="L48" s="7">
-        <v>1074</v>
-      </c>
+      <c r="D48" s="5"/>
+      <c r="E48" s="3"/>
+      <c r="F48" s="6"/>
+      <c r="G48" s="7"/>
+      <c r="H48" s="8"/>
+      <c r="I48" s="7"/>
+      <c r="J48" s="7"/>
+      <c r="K48" s="3"/>
+      <c r="L48" s="7"/>
     </row>
     <row r="49" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="inlineStr">
@@ -2923,33 +2189,15 @@
           <t>Xã Đức Phú</t>
         </is>
       </c>
-      <c r="D49" s="5">
-        <v>668</v>
-      </c>
-      <c r="E49" s="3">
-        <v>-100</v>
-      </c>
-      <c r="F49" s="6">
-        <v>568</v>
-      </c>
-      <c r="G49" s="7">
-        <v>557</v>
-      </c>
-      <c r="H49" s="3">
-        <v>-50</v>
-      </c>
-      <c r="I49" s="7">
-        <v>507</v>
-      </c>
-      <c r="J49" s="7">
-        <v>1091</v>
-      </c>
-      <c r="K49" s="3">
-        <v>-450</v>
-      </c>
-      <c r="L49" s="7">
-        <v>641</v>
-      </c>
+      <c r="D49" s="5"/>
+      <c r="E49" s="3"/>
+      <c r="F49" s="6"/>
+      <c r="G49" s="7"/>
+      <c r="H49" s="3"/>
+      <c r="I49" s="7"/>
+      <c r="J49" s="7"/>
+      <c r="K49" s="3"/>
+      <c r="L49" s="7"/>
     </row>
     <row r="50" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="inlineStr">
@@ -2967,31 +2215,15 @@
           <t>Phường Bàn Thạch</t>
         </is>
       </c>
-      <c r="D50" s="5">
-        <v>52</v>
-      </c>
-      <c r="E50" s="3">
-        <v>-5</v>
-      </c>
-      <c r="F50" s="6">
-        <v>47</v>
-      </c>
-      <c r="G50" s="7">
-        <v>245</v>
-      </c>
-      <c r="H50" s="3">
-        <v>-100</v>
-      </c>
-      <c r="I50" s="7">
-        <v>145</v>
-      </c>
-      <c r="J50" s="7">
-        <v>38</v>
-      </c>
+      <c r="D50" s="5"/>
+      <c r="E50" s="3"/>
+      <c r="F50" s="6"/>
+      <c r="G50" s="7"/>
+      <c r="H50" s="3"/>
+      <c r="I50" s="7"/>
+      <c r="J50" s="7"/>
       <c r="K50" s="20"/>
-      <c r="L50" s="7">
-        <v>38</v>
-      </c>
+      <c r="L50" s="7"/>
     </row>
     <row r="51" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="inlineStr">
@@ -3009,33 +2241,15 @@
           <t>Phường Hương Trà</t>
         </is>
       </c>
-      <c r="D51" s="5">
-        <v>41</v>
-      </c>
-      <c r="E51" s="3">
-        <v>-35</v>
-      </c>
-      <c r="F51" s="6">
-        <v>6</v>
-      </c>
-      <c r="G51" s="7">
-        <v>512</v>
-      </c>
-      <c r="H51" s="3">
-        <v>-200</v>
-      </c>
-      <c r="I51" s="7">
-        <v>312</v>
-      </c>
-      <c r="J51" s="7">
-        <v>285</v>
-      </c>
-      <c r="K51" s="10">
-        <v>-90</v>
-      </c>
-      <c r="L51" s="7">
-        <v>195</v>
-      </c>
+      <c r="D51" s="5"/>
+      <c r="E51" s="3"/>
+      <c r="F51" s="6"/>
+      <c r="G51" s="7"/>
+      <c r="H51" s="3"/>
+      <c r="I51" s="7"/>
+      <c r="J51" s="7"/>
+      <c r="K51" s="10"/>
+      <c r="L51" s="7"/>
     </row>
     <row r="52" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="inlineStr">
@@ -3053,29 +2267,15 @@
           <t>Phường Quảng Phú</t>
         </is>
       </c>
-      <c r="D52" s="5">
-        <v>0</v>
-      </c>
+      <c r="D52" s="5"/>
       <c r="E52" s="19"/>
-      <c r="F52" s="6">
-        <v>0</v>
-      </c>
-      <c r="G52" s="7">
-        <v>60</v>
-      </c>
-      <c r="H52" s="3">
-        <v>-30</v>
-      </c>
-      <c r="I52" s="7">
-        <v>30</v>
-      </c>
-      <c r="J52" s="7">
-        <v>3</v>
-      </c>
+      <c r="F52" s="6"/>
+      <c r="G52" s="7"/>
+      <c r="H52" s="3"/>
+      <c r="I52" s="7"/>
+      <c r="J52" s="7"/>
       <c r="K52" s="20"/>
-      <c r="L52" s="7">
-        <v>3</v>
-      </c>
+      <c r="L52" s="7"/>
     </row>
     <row r="53" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="inlineStr">
@@ -3093,31 +2293,15 @@
           <t>Phường Tam Kỳ</t>
         </is>
       </c>
-      <c r="D53" s="5">
-        <v>0</v>
-      </c>
+      <c r="D53" s="5"/>
       <c r="E53" s="19"/>
-      <c r="F53" s="6">
-        <v>0</v>
-      </c>
-      <c r="G53" s="7">
-        <v>210</v>
-      </c>
-      <c r="H53" s="3">
-        <v>-100</v>
-      </c>
-      <c r="I53" s="7">
-        <v>110</v>
-      </c>
-      <c r="J53" s="7">
-        <v>199</v>
-      </c>
-      <c r="K53" s="10">
-        <v>-5</v>
-      </c>
-      <c r="L53" s="7">
-        <v>194</v>
-      </c>
+      <c r="F53" s="6"/>
+      <c r="G53" s="7"/>
+      <c r="H53" s="3"/>
+      <c r="I53" s="7"/>
+      <c r="J53" s="7"/>
+      <c r="K53" s="10"/>
+      <c r="L53" s="7"/>
     </row>
     <row r="54" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="inlineStr">
@@ -3135,33 +2319,15 @@
           <t>Xã Tam Xuân</t>
         </is>
       </c>
-      <c r="D54" s="5">
-        <v>153</v>
-      </c>
-      <c r="E54" s="3">
-        <v>-35</v>
-      </c>
-      <c r="F54" s="6">
-        <v>118</v>
-      </c>
-      <c r="G54" s="7">
-        <v>84507</v>
-      </c>
-      <c r="H54" s="8">
-        <v>-19820</v>
-      </c>
-      <c r="I54" s="7">
-        <v>64687</v>
-      </c>
-      <c r="J54" s="7">
-        <v>3814</v>
-      </c>
-      <c r="K54" s="11">
-        <v>-1555</v>
-      </c>
-      <c r="L54" s="7">
-        <v>2259</v>
-      </c>
+      <c r="D54" s="5"/>
+      <c r="E54" s="3"/>
+      <c r="F54" s="6"/>
+      <c r="G54" s="7"/>
+      <c r="H54" s="8"/>
+      <c r="I54" s="7"/>
+      <c r="J54" s="7"/>
+      <c r="K54" s="11"/>
+      <c r="L54" s="7"/>
     </row>
     <row r="55" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="inlineStr">
@@ -3179,33 +2345,15 @@
           <t>Xã Lãnh Ngọc</t>
         </is>
       </c>
-      <c r="D55" s="5">
-        <v>1139</v>
-      </c>
-      <c r="E55" s="3">
-        <v>-200</v>
-      </c>
-      <c r="F55" s="6">
-        <v>939</v>
-      </c>
-      <c r="G55" s="7">
-        <v>35425</v>
-      </c>
-      <c r="H55" s="3">
-        <v>-400</v>
-      </c>
-      <c r="I55" s="7">
-        <v>35025</v>
-      </c>
-      <c r="J55" s="7">
-        <v>38627</v>
-      </c>
-      <c r="K55" s="8">
-        <v>-3500</v>
-      </c>
-      <c r="L55" s="7">
-        <v>35127</v>
-      </c>
+      <c r="D55" s="5"/>
+      <c r="E55" s="3"/>
+      <c r="F55" s="6"/>
+      <c r="G55" s="7"/>
+      <c r="H55" s="3"/>
+      <c r="I55" s="7"/>
+      <c r="J55" s="7"/>
+      <c r="K55" s="8"/>
+      <c r="L55" s="7"/>
     </row>
     <row r="56" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="inlineStr">
@@ -3223,33 +2371,15 @@
           <t>Xã Sơn Cẩm Hà</t>
         </is>
       </c>
-      <c r="D56" s="5">
-        <v>1534</v>
-      </c>
-      <c r="E56" s="3">
-        <v>-200</v>
-      </c>
-      <c r="F56" s="6">
-        <v>1334</v>
-      </c>
-      <c r="G56" s="7">
-        <v>36259</v>
-      </c>
-      <c r="H56" s="3">
-        <v>-200</v>
-      </c>
-      <c r="I56" s="7">
-        <v>36059</v>
-      </c>
-      <c r="J56" s="7">
-        <v>55838</v>
-      </c>
-      <c r="K56" s="8">
-        <v>-3500</v>
-      </c>
-      <c r="L56" s="7">
-        <v>52338</v>
-      </c>
+      <c r="D56" s="5"/>
+      <c r="E56" s="3"/>
+      <c r="F56" s="6"/>
+      <c r="G56" s="7"/>
+      <c r="H56" s="3"/>
+      <c r="I56" s="7"/>
+      <c r="J56" s="7"/>
+      <c r="K56" s="8"/>
+      <c r="L56" s="7"/>
     </row>
     <row r="57" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A57" s="3" t="inlineStr">
@@ -3267,33 +2397,15 @@
           <t>Xã Thạnh Bình</t>
         </is>
       </c>
-      <c r="D57" s="5">
-        <v>2086</v>
-      </c>
-      <c r="E57" s="3">
-        <v>-400</v>
-      </c>
-      <c r="F57" s="6">
-        <v>1686</v>
-      </c>
-      <c r="G57" s="7">
-        <v>38736</v>
-      </c>
-      <c r="H57" s="3">
-        <v>-400</v>
-      </c>
-      <c r="I57" s="7">
-        <v>38336</v>
-      </c>
-      <c r="J57" s="7">
-        <v>44790</v>
-      </c>
-      <c r="K57" s="8">
-        <v>-1522</v>
-      </c>
-      <c r="L57" s="7">
-        <v>43268</v>
-      </c>
+      <c r="D57" s="5"/>
+      <c r="E57" s="3"/>
+      <c r="F57" s="6"/>
+      <c r="G57" s="7"/>
+      <c r="H57" s="3"/>
+      <c r="I57" s="7"/>
+      <c r="J57" s="7"/>
+      <c r="K57" s="8"/>
+      <c r="L57" s="7"/>
     </row>
     <row r="58" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="inlineStr">
@@ -3311,33 +2423,15 @@
           <t>Xã Tiên Phước</t>
         </is>
       </c>
-      <c r="D58" s="5">
-        <v>1094</v>
-      </c>
-      <c r="E58" s="3">
-        <v>-151</v>
-      </c>
-      <c r="F58" s="6">
-        <v>943</v>
-      </c>
-      <c r="G58" s="7">
-        <v>27531</v>
-      </c>
-      <c r="H58" s="3">
-        <v>-500</v>
-      </c>
-      <c r="I58" s="7">
-        <v>27031</v>
-      </c>
-      <c r="J58" s="7">
-        <v>43234</v>
-      </c>
-      <c r="K58" s="8">
-        <v>-1600</v>
-      </c>
-      <c r="L58" s="7">
-        <v>41634</v>
-      </c>
+      <c r="D58" s="5"/>
+      <c r="E58" s="3"/>
+      <c r="F58" s="6"/>
+      <c r="G58" s="7"/>
+      <c r="H58" s="3"/>
+      <c r="I58" s="7"/>
+      <c r="J58" s="7"/>
+      <c r="K58" s="8"/>
+      <c r="L58" s="7"/>
     </row>
     <row r="59" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A59" s="3" t="inlineStr">
@@ -3355,27 +2449,15 @@
           <t>Phường Hội An</t>
         </is>
       </c>
-      <c r="D59" s="5">
-        <v>0</v>
-      </c>
+      <c r="D59" s="5"/>
       <c r="E59" s="19"/>
-      <c r="F59" s="6">
-        <v>0</v>
-      </c>
-      <c r="G59" s="7">
-        <v>0</v>
-      </c>
+      <c r="F59" s="6"/>
+      <c r="G59" s="7"/>
       <c r="H59" s="19"/>
-      <c r="I59" s="7">
-        <v>0</v>
-      </c>
-      <c r="J59" s="7">
-        <v>20</v>
-      </c>
+      <c r="I59" s="7"/>
+      <c r="J59" s="7"/>
       <c r="K59" s="19"/>
-      <c r="L59" s="7">
-        <v>20</v>
-      </c>
+      <c r="L59" s="7"/>
     </row>
     <row r="60" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A60" s="3" t="inlineStr">
@@ -3393,27 +2475,15 @@
           <t>Phường Hội An Tây</t>
         </is>
       </c>
-      <c r="D60" s="5">
-        <v>0</v>
-      </c>
+      <c r="D60" s="5"/>
       <c r="E60" s="19"/>
-      <c r="F60" s="6">
-        <v>0</v>
-      </c>
-      <c r="G60" s="7">
-        <v>0</v>
-      </c>
+      <c r="F60" s="6"/>
+      <c r="G60" s="7"/>
       <c r="H60" s="19"/>
-      <c r="I60" s="7">
-        <v>0</v>
-      </c>
-      <c r="J60" s="7">
-        <v>0</v>
-      </c>
+      <c r="I60" s="7"/>
+      <c r="J60" s="7"/>
       <c r="K60" s="19"/>
-      <c r="L60" s="7">
-        <v>0</v>
-      </c>
+      <c r="L60" s="7"/>
     </row>
     <row r="61" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A61" s="3" t="inlineStr">
@@ -3431,27 +2501,15 @@
           <t>Phường Hội An Đông</t>
         </is>
       </c>
-      <c r="D61" s="5">
-        <v>0</v>
-      </c>
+      <c r="D61" s="5"/>
       <c r="E61" s="19"/>
-      <c r="F61" s="6">
-        <v>0</v>
-      </c>
-      <c r="G61" s="7">
-        <v>18</v>
-      </c>
+      <c r="F61" s="6"/>
+      <c r="G61" s="7"/>
       <c r="H61" s="19"/>
-      <c r="I61" s="7">
-        <v>18</v>
-      </c>
-      <c r="J61" s="7">
-        <v>0</v>
-      </c>
+      <c r="I61" s="7"/>
+      <c r="J61" s="7"/>
       <c r="K61" s="19"/>
-      <c r="L61" s="7">
-        <v>0</v>
-      </c>
+      <c r="L61" s="7"/>
     </row>
     <row r="62" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A62" s="3" t="inlineStr">
@@ -3469,27 +2527,15 @@
           <t>Xã Tân Hiệp</t>
         </is>
       </c>
-      <c r="D62" s="5">
-        <v>0</v>
-      </c>
+      <c r="D62" s="5"/>
       <c r="E62" s="19"/>
-      <c r="F62" s="6">
-        <v>0</v>
-      </c>
-      <c r="G62" s="7">
-        <v>0</v>
-      </c>
+      <c r="F62" s="6"/>
+      <c r="G62" s="7"/>
       <c r="H62" s="19"/>
-      <c r="I62" s="7">
-        <v>0</v>
-      </c>
-      <c r="J62" s="7">
-        <v>0</v>
-      </c>
+      <c r="I62" s="7"/>
+      <c r="J62" s="7"/>
       <c r="K62" s="19"/>
-      <c r="L62" s="7">
-        <v>0</v>
-      </c>
+      <c r="L62" s="7"/>
     </row>
     <row r="63" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A63" s="3" t="inlineStr">
@@ -3507,33 +2553,15 @@
           <t>Xã Bến Giằng</t>
         </is>
       </c>
-      <c r="D63" s="5">
-        <v>29158</v>
-      </c>
-      <c r="E63" s="3">
-        <v>700</v>
-      </c>
-      <c r="F63" s="6">
-        <v>29858</v>
-      </c>
-      <c r="G63" s="7">
-        <v>6132</v>
-      </c>
-      <c r="H63" s="3">
-        <v>400</v>
-      </c>
-      <c r="I63" s="7">
-        <v>6532</v>
-      </c>
-      <c r="J63" s="7">
-        <v>4460</v>
-      </c>
-      <c r="K63" s="3">
-        <v>-400</v>
-      </c>
-      <c r="L63" s="7">
-        <v>4060</v>
-      </c>
+      <c r="D63" s="5"/>
+      <c r="E63" s="3"/>
+      <c r="F63" s="6"/>
+      <c r="G63" s="7"/>
+      <c r="H63" s="3"/>
+      <c r="I63" s="7"/>
+      <c r="J63" s="7"/>
+      <c r="K63" s="3"/>
+      <c r="L63" s="7"/>
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="inlineStr">
@@ -3551,33 +2579,15 @@
           <t>Xã La Dêê</t>
         </is>
       </c>
-      <c r="D64" s="5">
-        <v>11123</v>
-      </c>
-      <c r="E64" s="3">
-        <v>700</v>
-      </c>
-      <c r="F64" s="6">
-        <v>11823</v>
-      </c>
-      <c r="G64" s="7">
-        <v>268</v>
-      </c>
-      <c r="H64" s="3">
-        <v>300</v>
-      </c>
-      <c r="I64" s="7">
-        <v>568</v>
-      </c>
-      <c r="J64" s="7">
-        <v>3233</v>
-      </c>
-      <c r="K64" s="3">
-        <v>-544</v>
-      </c>
-      <c r="L64" s="7">
-        <v>2689</v>
-      </c>
+      <c r="D64" s="5"/>
+      <c r="E64" s="3"/>
+      <c r="F64" s="6"/>
+      <c r="G64" s="7"/>
+      <c r="H64" s="3"/>
+      <c r="I64" s="7"/>
+      <c r="J64" s="7"/>
+      <c r="K64" s="3"/>
+      <c r="L64" s="7"/>
     </row>
     <row r="65" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="inlineStr">
@@ -3595,33 +2605,15 @@
           <t>Xã La Êê</t>
         </is>
       </c>
-      <c r="D65" s="5">
-        <v>8727</v>
-      </c>
-      <c r="E65" s="3">
-        <v>600</v>
-      </c>
-      <c r="F65" s="6">
-        <v>9327</v>
-      </c>
-      <c r="G65" s="7">
-        <v>1906</v>
-      </c>
-      <c r="H65" s="3">
-        <v>300</v>
-      </c>
-      <c r="I65" s="7">
-        <v>2206</v>
-      </c>
-      <c r="J65" s="7">
-        <v>1382</v>
-      </c>
-      <c r="K65" s="3">
-        <v>-400</v>
-      </c>
-      <c r="L65" s="7">
-        <v>982</v>
-      </c>
+      <c r="D65" s="5"/>
+      <c r="E65" s="3"/>
+      <c r="F65" s="6"/>
+      <c r="G65" s="7"/>
+      <c r="H65" s="3"/>
+      <c r="I65" s="7"/>
+      <c r="J65" s="7"/>
+      <c r="K65" s="3"/>
+      <c r="L65" s="7"/>
     </row>
     <row r="66" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A66" s="3" t="inlineStr">
@@ -3639,33 +2631,15 @@
           <t>Xã Nam Giang</t>
         </is>
       </c>
-      <c r="D66" s="5">
-        <v>15267</v>
-      </c>
-      <c r="E66" s="3">
-        <v>700</v>
-      </c>
-      <c r="F66" s="6">
-        <v>15967</v>
-      </c>
-      <c r="G66" s="7">
-        <v>1010</v>
-      </c>
-      <c r="H66" s="3">
-        <v>300</v>
-      </c>
-      <c r="I66" s="7">
-        <v>1310</v>
-      </c>
-      <c r="J66" s="7">
-        <v>1288</v>
-      </c>
-      <c r="K66" s="3">
-        <v>-500</v>
-      </c>
-      <c r="L66" s="7">
-        <v>788</v>
-      </c>
+      <c r="D66" s="5"/>
+      <c r="E66" s="3"/>
+      <c r="F66" s="6"/>
+      <c r="G66" s="7"/>
+      <c r="H66" s="3"/>
+      <c r="I66" s="7"/>
+      <c r="J66" s="7"/>
+      <c r="K66" s="3"/>
+      <c r="L66" s="7"/>
     </row>
     <row r="67" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A67" s="3" t="inlineStr">
@@ -3683,33 +2657,15 @@
           <t>Xã Thạnh Mỹ</t>
         </is>
       </c>
-      <c r="D67" s="5">
-        <v>8872</v>
-      </c>
-      <c r="E67" s="3">
-        <v>700</v>
-      </c>
-      <c r="F67" s="6">
-        <v>9572</v>
-      </c>
-      <c r="G67" s="7">
-        <v>2893</v>
-      </c>
-      <c r="H67" s="3">
-        <v>400</v>
-      </c>
-      <c r="I67" s="7">
-        <v>3293</v>
-      </c>
-      <c r="J67" s="7">
-        <v>2864</v>
-      </c>
-      <c r="K67" s="3">
-        <v>-500</v>
-      </c>
-      <c r="L67" s="7">
-        <v>2364</v>
-      </c>
+      <c r="D67" s="5"/>
+      <c r="E67" s="3"/>
+      <c r="F67" s="6"/>
+      <c r="G67" s="7"/>
+      <c r="H67" s="3"/>
+      <c r="I67" s="7"/>
+      <c r="J67" s="7"/>
+      <c r="K67" s="3"/>
+      <c r="L67" s="7"/>
     </row>
     <row r="68" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A68" s="3" t="inlineStr">
@@ -3727,35 +2683,20 @@
           <t>Xã Đắc Pring</t>
         </is>
       </c>
-      <c r="D68" s="5">
-        <v>10003</v>
-      </c>
-      <c r="E68" s="3">
-        <v>600</v>
-      </c>
+      <c r="D68" s="5"/>
+      <c r="E68" s="3"/>
       <c r="F68" s="6">
         <f t="shared" ref="F68:F80" si="3">D68+E68</f>
-        <v>10603</v>
-      </c>
-      <c r="G68" s="7">
-        <v>1625</v>
-      </c>
-      <c r="H68" s="3">
-        <v>300</v>
-      </c>
+      </c>
+      <c r="G68" s="7"/>
+      <c r="H68" s="3"/>
       <c r="I68" s="7">
         <f t="shared" ref="I68:I80" si="4">G68+H68</f>
-        <v>1925</v>
-      </c>
-      <c r="J68" s="7">
-        <v>1146</v>
-      </c>
-      <c r="K68" s="3">
-        <v>-500</v>
-      </c>
+      </c>
+      <c r="J68" s="7"/>
+      <c r="K68" s="3"/>
       <c r="L68" s="7">
         <f t="shared" ref="L68:L80" si="5">J68+K68</f>
-        <v>646</v>
       </c>
     </row>
     <row r="69" spans="1:12" x14ac:dyDescent="0.25">
@@ -3774,33 +2715,15 @@
           <t>Xã Khâm Đức</t>
         </is>
       </c>
-      <c r="D69" s="5">
-        <v>15565</v>
-      </c>
-      <c r="E69" s="3">
-        <v>300</v>
-      </c>
-      <c r="F69" s="6">
-        <v>15865</v>
-      </c>
-      <c r="G69" s="7">
-        <v>6730</v>
-      </c>
-      <c r="H69" s="3">
-        <v>200</v>
-      </c>
-      <c r="I69" s="7">
-        <v>6930</v>
-      </c>
-      <c r="J69" s="7">
-        <v>5224</v>
-      </c>
-      <c r="K69" s="3">
-        <v>100</v>
-      </c>
-      <c r="L69" s="7">
-        <v>5324</v>
-      </c>
+      <c r="D69" s="5"/>
+      <c r="E69" s="3"/>
+      <c r="F69" s="6"/>
+      <c r="G69" s="7"/>
+      <c r="H69" s="3"/>
+      <c r="I69" s="7"/>
+      <c r="J69" s="7"/>
+      <c r="K69" s="3"/>
+      <c r="L69" s="7"/>
     </row>
     <row r="70" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A70" s="3" t="inlineStr">
@@ -3818,33 +2741,15 @@
           <t>Xã Phước Chánh</t>
         </is>
       </c>
-      <c r="D70" s="5">
-        <v>11955</v>
-      </c>
-      <c r="E70" s="3">
-        <v>300</v>
-      </c>
-      <c r="F70" s="6">
-        <v>12255</v>
-      </c>
-      <c r="G70" s="7">
-        <v>14208</v>
-      </c>
-      <c r="H70" s="3">
-        <v>200</v>
-      </c>
-      <c r="I70" s="7">
-        <v>14408</v>
-      </c>
-      <c r="J70" s="7">
-        <v>6213</v>
-      </c>
-      <c r="K70" s="3">
-        <v>100</v>
-      </c>
-      <c r="L70" s="7">
-        <v>6313</v>
-      </c>
+      <c r="D70" s="5"/>
+      <c r="E70" s="3"/>
+      <c r="F70" s="6"/>
+      <c r="G70" s="7"/>
+      <c r="H70" s="3"/>
+      <c r="I70" s="7"/>
+      <c r="J70" s="7"/>
+      <c r="K70" s="3"/>
+      <c r="L70" s="7"/>
     </row>
     <row r="71" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A71" s="3" t="inlineStr">
@@ -3862,33 +2767,15 @@
           <t>Xã Phước Hiệp</t>
         </is>
       </c>
-      <c r="D71" s="5">
-        <v>14219</v>
-      </c>
-      <c r="E71" s="3">
-        <v>300</v>
-      </c>
-      <c r="F71" s="6">
-        <v>14519</v>
-      </c>
-      <c r="G71" s="7">
-        <v>3830</v>
-      </c>
-      <c r="H71" s="3">
-        <v>200</v>
-      </c>
-      <c r="I71" s="7">
-        <v>4030</v>
-      </c>
-      <c r="J71" s="7">
-        <v>3869</v>
-      </c>
-      <c r="K71" s="3">
-        <v>100</v>
-      </c>
-      <c r="L71" s="7">
-        <v>3969</v>
-      </c>
+      <c r="D71" s="5"/>
+      <c r="E71" s="3"/>
+      <c r="F71" s="6"/>
+      <c r="G71" s="7"/>
+      <c r="H71" s="3"/>
+      <c r="I71" s="7"/>
+      <c r="J71" s="7"/>
+      <c r="K71" s="3"/>
+      <c r="L71" s="7"/>
     </row>
     <row r="72" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A72" s="3" t="inlineStr">
@@ -3906,33 +2793,15 @@
           <t>Xã Phước Năng</t>
         </is>
       </c>
-      <c r="D72" s="5">
-        <v>22304</v>
-      </c>
-      <c r="E72" s="3">
-        <v>300</v>
-      </c>
-      <c r="F72" s="6">
-        <v>22604</v>
-      </c>
-      <c r="G72" s="7">
-        <v>10228</v>
-      </c>
-      <c r="H72" s="3">
-        <v>200</v>
-      </c>
-      <c r="I72" s="7">
-        <v>10428</v>
-      </c>
-      <c r="J72" s="7">
-        <v>10994</v>
-      </c>
-      <c r="K72" s="3">
-        <v>100</v>
-      </c>
-      <c r="L72" s="7">
-        <v>11094</v>
-      </c>
+      <c r="D72" s="5"/>
+      <c r="E72" s="3"/>
+      <c r="F72" s="6"/>
+      <c r="G72" s="7"/>
+      <c r="H72" s="3"/>
+      <c r="I72" s="7"/>
+      <c r="J72" s="7"/>
+      <c r="K72" s="3"/>
+      <c r="L72" s="7"/>
     </row>
     <row r="73" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A73" s="3" t="inlineStr">
@@ -3950,33 +2819,15 @@
           <t>Xã Phước Thành</t>
         </is>
       </c>
-      <c r="D73" s="5">
-        <v>17113</v>
-      </c>
-      <c r="E73" s="3">
-        <v>300</v>
-      </c>
-      <c r="F73" s="6">
-        <v>17413</v>
-      </c>
-      <c r="G73" s="7">
-        <v>1372</v>
-      </c>
-      <c r="H73" s="3">
-        <v>200</v>
-      </c>
-      <c r="I73" s="7">
-        <v>1572</v>
-      </c>
-      <c r="J73" s="7">
-        <v>769</v>
-      </c>
-      <c r="K73" s="3">
-        <v>100</v>
-      </c>
-      <c r="L73" s="7">
-        <v>869</v>
-      </c>
+      <c r="D73" s="5"/>
+      <c r="E73" s="3"/>
+      <c r="F73" s="6"/>
+      <c r="G73" s="7"/>
+      <c r="H73" s="3"/>
+      <c r="I73" s="7"/>
+      <c r="J73" s="7"/>
+      <c r="K73" s="3"/>
+      <c r="L73" s="7"/>
     </row>
     <row r="74" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A74" s="3" t="inlineStr">
@@ -3994,33 +2845,15 @@
           <t>Xã Hiệp Đức</t>
         </is>
       </c>
-      <c r="D74" s="5">
-        <v>3133</v>
-      </c>
-      <c r="E74" s="8">
-        <v>-1000</v>
-      </c>
-      <c r="F74" s="6">
-        <v>2133</v>
-      </c>
-      <c r="G74" s="7">
-        <v>33539</v>
-      </c>
-      <c r="H74" s="8">
-        <v>-1500</v>
-      </c>
-      <c r="I74" s="7">
-        <v>32039</v>
-      </c>
-      <c r="J74" s="7">
-        <v>5028</v>
-      </c>
-      <c r="K74" s="8">
-        <v>-2000</v>
-      </c>
-      <c r="L74" s="7">
-        <v>3028</v>
-      </c>
+      <c r="D74" s="5"/>
+      <c r="E74" s="8"/>
+      <c r="F74" s="6"/>
+      <c r="G74" s="7"/>
+      <c r="H74" s="8"/>
+      <c r="I74" s="7"/>
+      <c r="J74" s="7"/>
+      <c r="K74" s="8"/>
+      <c r="L74" s="7"/>
     </row>
     <row r="75" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A75" s="3" t="inlineStr">
@@ -4038,29 +2871,15 @@
           <t>Xã Phước Trà</t>
         </is>
       </c>
-      <c r="D75" s="5">
-        <v>11033</v>
-      </c>
+      <c r="D75" s="5"/>
       <c r="E75" s="19"/>
-      <c r="F75" s="6">
-        <v>11033</v>
-      </c>
-      <c r="G75" s="7">
-        <v>5300</v>
-      </c>
+      <c r="F75" s="6"/>
+      <c r="G75" s="7"/>
       <c r="H75" s="19"/>
-      <c r="I75" s="7">
-        <v>5300</v>
-      </c>
-      <c r="J75" s="7">
-        <v>4828</v>
-      </c>
-      <c r="K75" s="8">
-        <v>-1000</v>
-      </c>
-      <c r="L75" s="7">
-        <v>3828</v>
-      </c>
+      <c r="I75" s="7"/>
+      <c r="J75" s="7"/>
+      <c r="K75" s="8"/>
+      <c r="L75" s="7"/>
     </row>
     <row r="76" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A76" s="3" t="inlineStr">
@@ -4078,33 +2897,15 @@
           <t>Xã Việt An</t>
         </is>
       </c>
-      <c r="D76" s="5">
-        <v>3037</v>
-      </c>
-      <c r="E76" s="8">
-        <v>-1000</v>
-      </c>
-      <c r="F76" s="6">
-        <v>2037</v>
-      </c>
-      <c r="G76" s="7">
-        <v>54109</v>
-      </c>
-      <c r="H76" s="8">
-        <v>-2500</v>
-      </c>
-      <c r="I76" s="7">
-        <v>51609</v>
-      </c>
-      <c r="J76" s="7">
-        <v>5160</v>
-      </c>
-      <c r="K76" s="8">
-        <v>-2000</v>
-      </c>
-      <c r="L76" s="7">
-        <v>3160</v>
-      </c>
+      <c r="D76" s="5"/>
+      <c r="E76" s="8"/>
+      <c r="F76" s="6"/>
+      <c r="G76" s="7"/>
+      <c r="H76" s="8"/>
+      <c r="I76" s="7"/>
+      <c r="J76" s="7"/>
+      <c r="K76" s="8"/>
+      <c r="L76" s="7"/>
     </row>
     <row r="77" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A77" s="3" t="inlineStr">
@@ -4122,33 +2923,15 @@
           <t>Xã Bến Hiên</t>
         </is>
       </c>
-      <c r="D77" s="5">
-        <v>19526</v>
-      </c>
-      <c r="E77" s="8">
-        <v>1843</v>
-      </c>
-      <c r="F77" s="6">
-        <v>21369</v>
-      </c>
-      <c r="G77" s="7">
-        <v>2421</v>
-      </c>
-      <c r="H77" s="8">
-        <v>1000</v>
-      </c>
-      <c r="I77" s="7">
-        <v>3421</v>
-      </c>
-      <c r="J77" s="7">
-        <v>2157</v>
-      </c>
-      <c r="K77" s="3">
-        <v>100</v>
-      </c>
-      <c r="L77" s="7">
-        <v>2257</v>
-      </c>
+      <c r="D77" s="5"/>
+      <c r="E77" s="8"/>
+      <c r="F77" s="6"/>
+      <c r="G77" s="7"/>
+      <c r="H77" s="8"/>
+      <c r="I77" s="7"/>
+      <c r="J77" s="7"/>
+      <c r="K77" s="3"/>
+      <c r="L77" s="7"/>
     </row>
     <row r="78" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A78" s="3" t="inlineStr">
@@ -4166,33 +2949,15 @@
           <t>Xã Sông Kôn</t>
         </is>
       </c>
-      <c r="D78" s="5">
-        <v>59165</v>
-      </c>
-      <c r="E78" s="8">
-        <v>2500</v>
-      </c>
-      <c r="F78" s="6">
-        <v>61665</v>
-      </c>
-      <c r="G78" s="7">
-        <v>7406</v>
-      </c>
-      <c r="H78" s="8">
-        <v>1500</v>
-      </c>
-      <c r="I78" s="7">
-        <v>8906</v>
-      </c>
-      <c r="J78" s="7">
-        <v>4199</v>
-      </c>
-      <c r="K78" s="3">
-        <v>400</v>
-      </c>
-      <c r="L78" s="7">
-        <v>4599</v>
-      </c>
+      <c r="D78" s="5"/>
+      <c r="E78" s="8"/>
+      <c r="F78" s="6"/>
+      <c r="G78" s="7"/>
+      <c r="H78" s="8"/>
+      <c r="I78" s="7"/>
+      <c r="J78" s="7"/>
+      <c r="K78" s="3"/>
+      <c r="L78" s="7"/>
     </row>
     <row r="79" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A79" s="3" t="inlineStr">
@@ -4210,33 +2975,15 @@
           <t>Xã Sông Vàng</t>
         </is>
       </c>
-      <c r="D79" s="5">
-        <v>19732</v>
-      </c>
-      <c r="E79" s="3">
-        <v>500</v>
-      </c>
-      <c r="F79" s="6">
-        <v>20232</v>
-      </c>
-      <c r="G79" s="7">
-        <v>11178</v>
-      </c>
-      <c r="H79" s="3">
-        <v>600</v>
-      </c>
-      <c r="I79" s="7">
-        <v>11778</v>
-      </c>
-      <c r="J79" s="7">
-        <v>2293</v>
-      </c>
-      <c r="K79" s="3">
-        <v>100</v>
-      </c>
-      <c r="L79" s="7">
-        <v>2393</v>
-      </c>
+      <c r="D79" s="5"/>
+      <c r="E79" s="3"/>
+      <c r="F79" s="6"/>
+      <c r="G79" s="7"/>
+      <c r="H79" s="3"/>
+      <c r="I79" s="7"/>
+      <c r="J79" s="7"/>
+      <c r="K79" s="3"/>
+      <c r="L79" s="7"/>
     </row>
     <row r="80" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A80" s="3" t="inlineStr">
@@ -4254,33 +3001,15 @@
           <t>Xã Đông Giang</t>
         </is>
       </c>
-      <c r="D80" s="5">
-        <v>41462</v>
-      </c>
-      <c r="E80" s="8">
-        <v>3000</v>
-      </c>
-      <c r="F80" s="6">
-        <v>44462</v>
-      </c>
-      <c r="G80" s="7">
-        <v>3252</v>
-      </c>
-      <c r="H80" s="8">
-        <v>1000</v>
-      </c>
-      <c r="I80" s="7">
-        <v>4252</v>
-      </c>
-      <c r="J80" s="7">
-        <v>2993</v>
-      </c>
-      <c r="K80" s="3">
-        <v>400</v>
-      </c>
-      <c r="L80" s="7">
-        <v>3393</v>
-      </c>
+      <c r="D80" s="5"/>
+      <c r="E80" s="8"/>
+      <c r="F80" s="6"/>
+      <c r="G80" s="7"/>
+      <c r="H80" s="8"/>
+      <c r="I80" s="7"/>
+      <c r="J80" s="7"/>
+      <c r="K80" s="3"/>
+      <c r="L80" s="7"/>
     </row>
     <row r="81" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A81" s="12" t="inlineStr">

</xml_diff>